<commit_message>
Attempt on fixing issue that new renewable technologies are not linked with commodity fractions
</commit_message>
<xml_diff>
--- a/SubRES_TMPL/SubRES_NewTechs_Trans.xlsx
+++ b/SubRES_TMPL/SubRES_NewTechs_Trans.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\SubRES_TMPL\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AEB4CBCC-1696-4D76-8796-0E1E934CED66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6CC8EF5-1085-4DDE-9B2A-D76885AAC1EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="AVA" sheetId="18" r:id="rId1"/>
@@ -124,7 +124,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="24">
   <si>
     <t>~TFM_INS</t>
   </si>
@@ -193,6 +193,9 @@
   </si>
   <si>
     <t>REG1</t>
+  </si>
+  <si>
+    <t>*</t>
   </si>
 </sst>
 </file>
@@ -702,6 +705,14 @@
         <v>21</v>
       </c>
     </row>
+    <row r="5" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C5">
+        <v>1</v>
+      </c>
+    </row>
     <row r="6" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B6" s="11"/>
     </row>

</xml_diff>